<commit_message>
Update C61 - Document Planification 2222.xlsx
</commit_message>
<xml_diff>
--- a/docs/sprint1/C61 - Document Planification 2222.xlsx
+++ b/docs/sprint1/C61 - Document Planification 2222.xlsx
@@ -4,17 +4,16 @@
   <workbookPr date1904="0"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView xWindow="360" yWindow="15" windowWidth="20955" windowHeight="9720" activeTab="1" showHorizontalScroll="1" showVerticalScroll="1"/>
+    <workbookView xWindow="360" yWindow="15" windowWidth="20955" windowHeight="9720" activeTab="6" showHorizontalScroll="1" showVerticalScroll="1"/>
   </bookViews>
   <sheets>
     <sheet name="Planification" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="Planification Finale" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Sheet1" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Sprint 1" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="Sprint 2" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="Mi-mandat" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="Sprint 3" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet name="Sprint 4" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="Sprint 1" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Sprint 2" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Mi-mandat" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Sprint 3" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="Sprint 4" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
   <calcPr refMode="A1" iterate="0" iterateCount="100" iterateDelta="0.0001"/>
   <extLst>
@@ -24,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="166" uniqueCount="166">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="174" uniqueCount="174">
   <si>
     <t xml:space="preserve">Planification globale</t>
   </si>
@@ -522,6 +521,30 @@
   </si>
   <si>
     <t xml:space="preserve">Semaine D</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Création d'une Machine états générique C#</t>
+  </si>
+  <si>
+    <t>JM</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Assisté avec IA pour trouver les génériques de csharp, mais basé sur la conception FSM du cours de Jean-Christophe, avec un twist pour enlever les conditions</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Créer le template pour la machine de jeu entière</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Basé sur figure 5 du document de conception finale</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Créer le template pour la machine de jeu (environnement 3D)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Créer le template pour la fsm de victoire</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Gérer les liens entre les fsm</t>
   </si>
 </sst>
 </file>
@@ -550,13 +573,11 @@
     </font>
     <font>
       <sz val="11.000000"/>
-      <color indexed="64"/>
       <name val="Arial"/>
     </font>
     <font>
       <b/>
       <sz val="11.000000"/>
-      <color indexed="64"/>
       <name val="Arial"/>
     </font>
     <font>
@@ -566,12 +587,10 @@
     </font>
     <font>
       <sz val="11.000000"/>
-      <color indexed="64"/>
       <name val="Calibri"/>
     </font>
     <font>
       <sz val="36.000000"/>
-      <color indexed="64"/>
       <name val="Calibri"/>
     </font>
     <font>
@@ -581,13 +600,11 @@
     </font>
     <font>
       <sz val="16.000000"/>
-      <color indexed="64"/>
       <name val="Calibri"/>
     </font>
     <font>
       <i/>
       <sz val="9.000000"/>
-      <color indexed="64"/>
       <name val="Arial"/>
     </font>
     <font>
@@ -621,7 +638,6 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor indexed="64"/>
         <bgColor indexed="58"/>
       </patternFill>
     </fill>
@@ -713,7 +729,7 @@
     <xf fontId="1" fillId="0" borderId="0" numFmtId="42" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="0" applyProtection="0"/>
     <xf fontId="1" fillId="0" borderId="0" numFmtId="9" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="41">
+  <cellXfs count="43">
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0" applyProtection="0">
       <protection hidden="0" locked="1"/>
     </xf>
@@ -844,10 +860,18 @@
     <xf fontId="0" fillId="0" borderId="6" numFmtId="0" xfId="0" applyBorder="1" applyProtection="0">
       <protection hidden="0" locked="1"/>
     </xf>
-    <xf fontId="0" fillId="0" borderId="3" numFmtId="0" xfId="0" applyBorder="1" applyProtection="0">
+    <xf fontId="7" fillId="0" borderId="3" numFmtId="0" xfId="0" applyFont="1" applyBorder="1" applyProtection="0">
       <protection hidden="0" locked="1"/>
     </xf>
-    <xf fontId="0" fillId="0" borderId="4" numFmtId="0" xfId="0" applyBorder="1" applyProtection="0">
+    <xf fontId="7" fillId="0" borderId="4" numFmtId="0" xfId="0" applyFont="1" applyBorder="1" applyProtection="0">
+      <protection hidden="0" locked="1"/>
+    </xf>
+    <xf fontId="7" fillId="0" borderId="4" numFmtId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="0">
+      <alignment wrapText="1"/>
+      <protection hidden="0" locked="1"/>
+    </xf>
+    <xf fontId="7" fillId="0" borderId="0" numFmtId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="0">
+      <alignment wrapText="1"/>
       <protection hidden="0" locked="1"/>
     </xf>
   </cellXfs>
@@ -3357,7 +3381,7 @@
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{CCE6A557-97BC-4b89-ADB6-D9C93CAAB3DF}">
       <x14:dataValidations xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" count="3" disablePrompts="0">
-        <x14:dataValidation xr:uid="{00C10025-009E-4244-9B57-007800790052}" type="list" allowBlank="1" errorStyle="stop" imeMode="noControl" operator="between" showDropDown="0" showErrorMessage="1" showInputMessage="0">
+        <x14:dataValidation xr:uid="{00D90074-00E5-461C-A3DF-0091009D0056}" type="list" allowBlank="1" errorStyle="stop" imeMode="noControl" operator="between" showDropDown="0" showErrorMessage="1" showInputMessage="0">
           <x14:formula1>
             <xm:f>"Indispensable,Souhaitable,Optionnel"</xm:f>
           </x14:formula1>
@@ -3366,7 +3390,7 @@
           </x14:formula2>
           <xm:sqref>D6:D101</xm:sqref>
         </x14:dataValidation>
-        <x14:dataValidation xr:uid="{007400C6-00C2-46F8-998B-00F900B60092}" type="list" allowBlank="1" errorStyle="stop" imeMode="noControl" operator="between" showDropDown="0" showErrorMessage="1" showInputMessage="0">
+        <x14:dataValidation xr:uid="{005D00F6-00EF-4BD1-B2B4-004200020094}" type="list" allowBlank="1" errorStyle="stop" imeMode="noControl" operator="between" showDropDown="0" showErrorMessage="1" showInputMessage="0">
           <x14:formula1>
             <xm:f>"Sprint 1,Sprint 2,Sprint 3,Sprint 4"</xm:f>
           </x14:formula1>
@@ -3375,7 +3399,7 @@
           </x14:formula2>
           <xm:sqref>C6:C101</xm:sqref>
         </x14:dataValidation>
-        <x14:dataValidation xr:uid="{00BF0047-003B-4699-BC27-0068002300ED}" type="list" allowBlank="1" errorStyle="stop" imeMode="noControl" operator="between" showDropDown="0" showErrorMessage="1" showInputMessage="0">
+        <x14:dataValidation xr:uid="{001F009D-00F1-40FA-B029-009C008C00BC}" type="list" allowBlank="1" errorStyle="stop" imeMode="noControl" operator="between" showDropDown="0" showErrorMessage="1" showInputMessage="0">
           <x14:formula1>
             <xm:f>"3D,Les deux,NET"</xm:f>
           </x14:formula1>
@@ -3392,7 +3416,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac">
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="14.25"/>
   <cols>
     <col bestFit="1" customWidth="1" min="2" max="2" width="80.7109375"/>
     <col customWidth="1" min="3" max="9" width="28.140625"/>
@@ -3413,6 +3437,9 @@
       </c>
     </row>
     <row r="7">
+      <c r="A7">
+        <v>1</v>
+      </c>
       <c r="B7" s="13" t="s">
         <v>66</v>
       </c>
@@ -3423,6 +3450,9 @@
       <c r="E7" s="13"/>
     </row>
     <row r="8">
+      <c r="A8">
+        <v>2</v>
+      </c>
       <c r="B8" s="13" t="s">
         <v>68</v>
       </c>
@@ -3433,6 +3463,9 @@
       <c r="E8" s="13"/>
     </row>
     <row r="9">
+      <c r="A9">
+        <v>3</v>
+      </c>
       <c r="B9" s="13" t="s">
         <v>69</v>
       </c>
@@ -3441,6 +3474,9 @@
       <c r="E9" s="13"/>
     </row>
     <row r="10">
+      <c r="A10">
+        <v>4</v>
+      </c>
       <c r="B10" s="13" t="s">
         <v>70</v>
       </c>
@@ -3449,6 +3485,9 @@
       <c r="E10" s="13"/>
     </row>
     <row r="11">
+      <c r="A11">
+        <v>5</v>
+      </c>
       <c r="B11" s="13" t="s">
         <v>71</v>
       </c>
@@ -3457,6 +3496,9 @@
       <c r="E11" s="13"/>
     </row>
     <row r="12">
+      <c r="A12">
+        <v>6</v>
+      </c>
       <c r="B12" s="13" t="s">
         <v>72</v>
       </c>
@@ -3467,6 +3509,9 @@
       <c r="E12" s="13"/>
     </row>
     <row r="13">
+      <c r="A13">
+        <v>7</v>
+      </c>
       <c r="B13" s="13" t="s">
         <v>74</v>
       </c>
@@ -3477,138 +3522,207 @@
       <c r="E13" s="13"/>
     </row>
     <row r="14">
+      <c r="A14" s="14">
+        <v>8</v>
+      </c>
       <c r="B14" s="13"/>
       <c r="C14" s="13"/>
       <c r="D14" s="13"/>
       <c r="E14" s="13"/>
     </row>
     <row r="15">
+      <c r="A15" s="14">
+        <v>9</v>
+      </c>
       <c r="B15" s="13"/>
       <c r="C15" s="13"/>
       <c r="D15" s="13"/>
       <c r="E15" s="13"/>
     </row>
     <row r="16">
+      <c r="A16" s="14">
+        <v>10</v>
+      </c>
       <c r="B16" s="13"/>
       <c r="C16" s="13"/>
       <c r="D16" s="13"/>
       <c r="E16" s="13"/>
     </row>
     <row r="17">
+      <c r="A17" s="14">
+        <v>11</v>
+      </c>
       <c r="B17" s="13"/>
       <c r="C17" s="13"/>
       <c r="D17" s="13"/>
       <c r="E17" s="13"/>
     </row>
     <row r="18">
+      <c r="A18" s="14">
+        <v>12</v>
+      </c>
       <c r="B18" s="13"/>
       <c r="C18" s="13"/>
       <c r="D18" s="13"/>
       <c r="E18" s="13"/>
     </row>
     <row r="19">
+      <c r="A19" s="14">
+        <v>13</v>
+      </c>
       <c r="B19" s="13"/>
       <c r="C19" s="13"/>
       <c r="D19" s="13"/>
       <c r="E19" s="13"/>
     </row>
     <row r="20">
+      <c r="A20" s="14">
+        <v>14</v>
+      </c>
       <c r="B20" s="13"/>
       <c r="C20" s="13"/>
       <c r="D20" s="13"/>
       <c r="E20" s="13"/>
     </row>
     <row r="21">
+      <c r="A21" s="14">
+        <v>15</v>
+      </c>
       <c r="B21" s="13"/>
       <c r="C21" s="13"/>
       <c r="D21" s="13"/>
       <c r="E21" s="13"/>
     </row>
     <row r="22">
+      <c r="A22" s="14">
+        <v>16</v>
+      </c>
       <c r="B22" s="13"/>
       <c r="C22" s="13"/>
       <c r="D22" s="13"/>
       <c r="E22" s="13"/>
     </row>
     <row r="23">
+      <c r="A23" s="14">
+        <v>17</v>
+      </c>
       <c r="B23" s="13"/>
       <c r="C23" s="13"/>
       <c r="D23" s="13"/>
       <c r="E23" s="13"/>
     </row>
     <row r="24">
+      <c r="A24" s="14">
+        <v>18</v>
+      </c>
       <c r="B24" s="13"/>
       <c r="C24" s="13"/>
       <c r="D24" s="13"/>
       <c r="E24" s="13"/>
     </row>
     <row r="25">
+      <c r="A25" s="14">
+        <v>19</v>
+      </c>
       <c r="B25" s="13"/>
       <c r="C25" s="13"/>
       <c r="D25" s="13"/>
       <c r="E25" s="13"/>
     </row>
     <row r="26">
+      <c r="A26" s="14">
+        <v>20</v>
+      </c>
       <c r="B26" s="13"/>
       <c r="C26" s="13"/>
       <c r="D26" s="13"/>
       <c r="E26" s="13"/>
     </row>
     <row r="27">
+      <c r="A27" s="14">
+        <v>21</v>
+      </c>
       <c r="B27" s="13"/>
       <c r="C27" s="13"/>
       <c r="D27" s="13"/>
       <c r="E27" s="13"/>
     </row>
     <row r="28">
+      <c r="A28" s="14">
+        <v>22</v>
+      </c>
       <c r="B28" s="13"/>
       <c r="C28" s="13"/>
       <c r="D28" s="13"/>
       <c r="E28" s="13"/>
     </row>
     <row r="29">
+      <c r="A29" s="14">
+        <v>23</v>
+      </c>
       <c r="B29" s="13"/>
       <c r="C29" s="13"/>
       <c r="D29" s="13"/>
       <c r="E29" s="13"/>
     </row>
     <row r="30">
+      <c r="A30" s="14">
+        <v>24</v>
+      </c>
       <c r="B30" s="13"/>
       <c r="C30" s="13"/>
       <c r="D30" s="13"/>
       <c r="E30" s="13"/>
     </row>
     <row r="31">
+      <c r="A31" s="14">
+        <v>25</v>
+      </c>
       <c r="B31" s="13"/>
       <c r="C31" s="13"/>
       <c r="D31" s="13"/>
       <c r="E31" s="13"/>
     </row>
     <row r="32">
+      <c r="A32" s="14">
+        <v>26</v>
+      </c>
       <c r="B32" s="13"/>
       <c r="C32" s="13"/>
       <c r="D32" s="13"/>
       <c r="E32" s="13"/>
     </row>
     <row r="33">
+      <c r="A33" s="14">
+        <v>27</v>
+      </c>
       <c r="B33" s="13"/>
       <c r="C33" s="13"/>
       <c r="D33" s="13"/>
       <c r="E33" s="13"/>
     </row>
     <row r="34">
+      <c r="A34" s="14">
+        <v>28</v>
+      </c>
       <c r="B34" s="13"/>
       <c r="C34" s="13"/>
       <c r="D34" s="13"/>
       <c r="E34" s="13"/>
     </row>
     <row r="35">
+      <c r="A35" s="14">
+        <v>29</v>
+      </c>
       <c r="B35" s="13"/>
       <c r="C35" s="13"/>
       <c r="D35" s="13"/>
       <c r="E35" s="13"/>
     </row>
     <row r="36">
+      <c r="A36" s="14">
+        <v>30</v>
+      </c>
       <c r="B36" s="13"/>
       <c r="C36" s="13"/>
       <c r="D36" s="13"/>
@@ -5891,17 +6005,6 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac">
-  <sheetFormatPr defaultRowHeight="15"/>
-  <sheetData/>
-  <printOptions headings="0" gridLines="0"/>
-  <pageMargins left="0.70078740157480324" right="0.70078740157480324" top="0.75196850393700787" bottom="0.75196850393700787" header="0.29999999999999999" footer="0.29999999999999999"/>
-  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" usePrinterDefaults="1" blackAndWhite="0" draft="0" cellComments="none" useFirstPageNumber="0" errors="displayed" horizontalDpi="600" verticalDpi="600" copies="1"/>
-  <headerFooter/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac">
   <sheetPr filterMode="0">
     <outlinePr applyStyles="0" summaryBelow="1" summaryRight="1" showOutlineSymbols="1"/>
@@ -7938,7 +8041,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac">
   <sheetPr filterMode="0">
     <outlinePr applyStyles="0" summaryBelow="1" summaryRight="1" showOutlineSymbols="1"/>
@@ -9672,7 +9775,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac">
   <sheetPr filterMode="0">
     <outlinePr applyStyles="0" summaryBelow="1" summaryRight="1" showOutlineSymbols="1"/>
@@ -11292,7 +11395,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac">
   <sheetPr filterMode="0">
     <outlinePr applyStyles="0" summaryBelow="1" summaryRight="1" showOutlineSymbols="1"/>
@@ -13038,7 +13141,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac">
   <sheetPr filterMode="0">
     <outlinePr applyStyles="0" summaryBelow="1" summaryRight="1" showOutlineSymbols="1"/>
@@ -13047,11 +13150,11 @@
   <sheetFormatPr defaultColWidth="14.453125" defaultRowHeight="15" customHeight="1"/>
   <cols>
     <col customWidth="1" min="1" max="1" style="0" width="1.73"/>
-    <col customWidth="1" min="2" max="2" style="0" width="10.73"/>
+    <col customWidth="1" min="2" max="2" style="0" width="53.8515625"/>
     <col customWidth="1" min="3" max="3" style="0" width="17.73"/>
     <col customWidth="1" min="4" max="4" style="0" width="16.27"/>
     <col customWidth="1" min="5" max="5" style="0" width="15.539999999999999"/>
-    <col customWidth="1" min="6" max="6" style="0" width="20.27"/>
+    <col customWidth="1" min="6" max="6" style="0" width="37.28125"/>
     <col customWidth="1" min="7" max="7" style="0" width="10.73"/>
     <col customWidth="1" min="8" max="8" style="0" width="16.73"/>
     <col customWidth="1" min="9" max="9" style="0" width="20.449999999999999"/>
@@ -13064,12 +13167,12 @@
     <col customWidth="1" min="16" max="26" style="0" width="10.73"/>
   </cols>
   <sheetData>
-    <row r="1" ht="43.299999999999997">
+    <row r="1" ht="45">
       <c r="B1" s="1" t="s">
         <v>52</v>
       </c>
     </row>
-    <row r="3" ht="19.699999999999999">
+    <row r="3" ht="21">
       <c r="B3" s="21"/>
       <c r="C3" s="22"/>
       <c r="D3" s="22" t="s">
@@ -13093,7 +13196,7 @@
       <c r="N3" s="22"/>
       <c r="O3" s="23"/>
     </row>
-    <row r="4" ht="19.699999999999999">
+    <row r="4" ht="21">
       <c r="B4" s="21" t="s">
         <v>2</v>
       </c>
@@ -13138,314 +13241,1383 @@
       </c>
     </row>
     <row r="5" ht="15">
-      <c r="B5" s="39"/>
+      <c r="B5" s="39" t="s">
+        <v>66</v>
+      </c>
       <c r="C5" s="40"/>
+      <c r="D5" s="14"/>
+      <c r="E5" s="14"/>
       <c r="F5" s="40"/>
+      <c r="G5" s="14"/>
+      <c r="H5" s="14"/>
       <c r="I5" s="40"/>
+      <c r="J5" s="14"/>
+      <c r="K5" s="14"/>
       <c r="L5" s="40"/>
+      <c r="M5" s="14"/>
+      <c r="N5" s="14"/>
       <c r="O5" s="40"/>
-    </row>
-    <row r="6" ht="15">
-      <c r="B6" s="39"/>
-      <c r="C6" s="40"/>
-      <c r="F6" s="40"/>
+      <c r="P5" s="14"/>
+      <c r="Q5" s="14"/>
+      <c r="R5" s="14"/>
+      <c r="S5" s="14"/>
+      <c r="T5" s="14"/>
+      <c r="U5" s="14"/>
+      <c r="V5" s="14"/>
+      <c r="W5" s="14"/>
+      <c r="X5" s="14"/>
+      <c r="Y5" s="14"/>
+      <c r="Z5" s="14"/>
+    </row>
+    <row r="6" ht="57">
+      <c r="B6" s="39" t="s">
+        <v>166</v>
+      </c>
+      <c r="C6" s="40" t="s">
+        <v>167</v>
+      </c>
+      <c r="D6" s="14">
+        <v>1.5</v>
+      </c>
+      <c r="E6" s="14"/>
+      <c r="F6" s="41" t="s">
+        <v>168</v>
+      </c>
+      <c r="G6" s="14"/>
+      <c r="H6" s="14"/>
       <c r="I6" s="40"/>
+      <c r="J6" s="14"/>
+      <c r="K6" s="14"/>
       <c r="L6" s="40"/>
+      <c r="M6" s="14"/>
+      <c r="N6" s="14"/>
       <c r="O6" s="40"/>
-    </row>
-    <row r="7" ht="15">
-      <c r="B7" s="39"/>
+      <c r="P6" s="14"/>
+      <c r="Q6" s="14"/>
+      <c r="R6" s="14"/>
+      <c r="S6" s="14"/>
+      <c r="T6" s="14"/>
+      <c r="U6" s="14"/>
+      <c r="V6" s="14"/>
+      <c r="W6" s="14"/>
+      <c r="X6" s="14"/>
+      <c r="Y6" s="14"/>
+      <c r="Z6" s="14"/>
+    </row>
+    <row r="7" ht="28.5">
+      <c r="B7" s="39" t="s">
+        <v>169</v>
+      </c>
       <c r="C7" s="40"/>
-      <c r="F7" s="40"/>
+      <c r="D7" s="14">
+        <v>0.20000000000000001</v>
+      </c>
+      <c r="E7" s="14"/>
+      <c r="F7" s="41" t="s">
+        <v>170</v>
+      </c>
+      <c r="G7" s="14"/>
+      <c r="H7" s="14"/>
       <c r="I7" s="40"/>
+      <c r="J7" s="14"/>
+      <c r="K7" s="14"/>
       <c r="L7" s="40"/>
+      <c r="M7" s="14"/>
+      <c r="N7" s="14"/>
       <c r="O7" s="40"/>
+      <c r="P7" s="14"/>
+      <c r="Q7" s="14"/>
+      <c r="R7" s="14"/>
+      <c r="S7" s="14"/>
+      <c r="T7" s="14"/>
+      <c r="U7" s="14"/>
+      <c r="V7" s="14"/>
+      <c r="W7" s="14"/>
+      <c r="X7" s="14"/>
+      <c r="Y7" s="14"/>
+      <c r="Z7" s="14"/>
     </row>
     <row r="8" ht="15">
-      <c r="B8" s="39"/>
+      <c r="B8" s="39" t="s">
+        <v>171</v>
+      </c>
       <c r="C8" s="40"/>
-      <c r="F8" s="40"/>
+      <c r="D8" s="14">
+        <v>0.20000000000000001</v>
+      </c>
+      <c r="E8" s="14"/>
+      <c r="F8" s="41"/>
+      <c r="G8" s="14"/>
+      <c r="H8" s="14"/>
       <c r="I8" s="40"/>
+      <c r="J8" s="14"/>
+      <c r="K8" s="14"/>
       <c r="L8" s="40"/>
+      <c r="M8" s="14"/>
+      <c r="N8" s="14"/>
       <c r="O8" s="40"/>
+      <c r="P8" s="14"/>
+      <c r="Q8" s="14"/>
+      <c r="R8" s="14"/>
+      <c r="S8" s="14"/>
+      <c r="T8" s="14"/>
+      <c r="U8" s="14"/>
+      <c r="V8" s="14"/>
+      <c r="W8" s="14"/>
+      <c r="X8" s="14"/>
+      <c r="Y8" s="14"/>
+      <c r="Z8" s="14"/>
     </row>
     <row r="9" ht="15">
-      <c r="B9" s="39"/>
+      <c r="B9" s="39" t="s">
+        <v>172</v>
+      </c>
       <c r="C9" s="40"/>
-      <c r="F9" s="40"/>
+      <c r="D9" s="14">
+        <v>0.20000000000000001</v>
+      </c>
+      <c r="E9" s="14"/>
+      <c r="F9" s="41"/>
+      <c r="G9" s="14"/>
+      <c r="H9" s="14"/>
       <c r="I9" s="40"/>
+      <c r="J9" s="14"/>
+      <c r="K9" s="14"/>
       <c r="L9" s="40"/>
+      <c r="M9" s="14"/>
+      <c r="N9" s="14"/>
       <c r="O9" s="40"/>
+      <c r="P9" s="14"/>
+      <c r="Q9" s="14"/>
+      <c r="R9" s="14"/>
+      <c r="S9" s="14"/>
+      <c r="T9" s="14"/>
+      <c r="U9" s="14"/>
+      <c r="V9" s="14"/>
+      <c r="W9" s="14"/>
+      <c r="X9" s="14"/>
+      <c r="Y9" s="14"/>
+      <c r="Z9" s="14"/>
     </row>
     <row r="10" ht="15">
-      <c r="B10" s="39"/>
+      <c r="B10" s="39" t="s">
+        <v>173</v>
+      </c>
       <c r="C10" s="40"/>
-      <c r="F10" s="40"/>
+      <c r="D10" s="14">
+        <v>0.5</v>
+      </c>
+      <c r="E10" s="14"/>
+      <c r="F10" s="41"/>
+      <c r="G10" s="14"/>
+      <c r="H10" s="14"/>
       <c r="I10" s="40"/>
+      <c r="J10" s="14"/>
+      <c r="K10" s="14"/>
       <c r="L10" s="40"/>
+      <c r="M10" s="14"/>
+      <c r="N10" s="14"/>
       <c r="O10" s="40"/>
+      <c r="P10" s="14"/>
+      <c r="Q10" s="14"/>
+      <c r="R10" s="14"/>
+      <c r="S10" s="14"/>
+      <c r="T10" s="14"/>
+      <c r="U10" s="14"/>
+      <c r="V10" s="14"/>
+      <c r="W10" s="14"/>
+      <c r="X10" s="14"/>
+      <c r="Y10" s="14"/>
+      <c r="Z10" s="14"/>
     </row>
     <row r="11" ht="15">
       <c r="B11" s="39"/>
       <c r="C11" s="40"/>
-      <c r="F11" s="40"/>
+      <c r="D11" s="14"/>
+      <c r="E11" s="14"/>
+      <c r="F11" s="41"/>
+      <c r="G11" s="14"/>
+      <c r="H11" s="14"/>
       <c r="I11" s="40"/>
+      <c r="J11" s="14"/>
+      <c r="K11" s="14"/>
       <c r="L11" s="40"/>
+      <c r="M11" s="14"/>
+      <c r="N11" s="14"/>
       <c r="O11" s="40"/>
+      <c r="P11" s="14"/>
+      <c r="Q11" s="14"/>
+      <c r="R11" s="14"/>
+      <c r="S11" s="14"/>
+      <c r="T11" s="14"/>
+      <c r="U11" s="14"/>
+      <c r="V11" s="14"/>
+      <c r="W11" s="14"/>
+      <c r="X11" s="14"/>
+      <c r="Y11" s="14"/>
+      <c r="Z11" s="14"/>
     </row>
     <row r="12" ht="15">
       <c r="B12" s="39"/>
       <c r="C12" s="40"/>
-      <c r="F12" s="40"/>
+      <c r="D12" s="14"/>
+      <c r="E12" s="14"/>
+      <c r="F12" s="41"/>
+      <c r="G12" s="14"/>
+      <c r="H12" s="14"/>
       <c r="I12" s="40"/>
+      <c r="J12" s="14"/>
+      <c r="K12" s="14"/>
       <c r="L12" s="40"/>
+      <c r="M12" s="14"/>
+      <c r="N12" s="14"/>
       <c r="O12" s="40"/>
+      <c r="P12" s="14"/>
+      <c r="Q12" s="14"/>
+      <c r="R12" s="14"/>
+      <c r="S12" s="14"/>
+      <c r="T12" s="14"/>
+      <c r="U12" s="14"/>
+      <c r="V12" s="14"/>
+      <c r="W12" s="14"/>
+      <c r="X12" s="14"/>
+      <c r="Y12" s="14"/>
+      <c r="Z12" s="14"/>
     </row>
     <row r="13" ht="15">
       <c r="B13" s="39"/>
       <c r="C13" s="40"/>
-      <c r="F13" s="40"/>
+      <c r="D13" s="14"/>
+      <c r="E13" s="14"/>
+      <c r="F13" s="41"/>
+      <c r="G13" s="14"/>
+      <c r="H13" s="14"/>
       <c r="I13" s="40"/>
+      <c r="J13" s="14"/>
+      <c r="K13" s="14"/>
       <c r="L13" s="40"/>
+      <c r="M13" s="14"/>
+      <c r="N13" s="14"/>
       <c r="O13" s="40"/>
+      <c r="P13" s="14"/>
+      <c r="Q13" s="14"/>
+      <c r="R13" s="14"/>
+      <c r="S13" s="14"/>
+      <c r="T13" s="14"/>
+      <c r="U13" s="14"/>
+      <c r="V13" s="14"/>
+      <c r="W13" s="14"/>
+      <c r="X13" s="14"/>
+      <c r="Y13" s="14"/>
+      <c r="Z13" s="14"/>
     </row>
     <row r="14" ht="15">
       <c r="B14" s="39"/>
       <c r="C14" s="40"/>
-      <c r="F14" s="40"/>
+      <c r="D14" s="14"/>
+      <c r="E14" s="14"/>
+      <c r="F14" s="41"/>
+      <c r="G14" s="14"/>
+      <c r="H14" s="14"/>
       <c r="I14" s="40"/>
+      <c r="J14" s="14"/>
+      <c r="K14" s="14"/>
       <c r="L14" s="40"/>
+      <c r="M14" s="14"/>
+      <c r="N14" s="14"/>
       <c r="O14" s="40"/>
+      <c r="P14" s="14"/>
+      <c r="Q14" s="14"/>
+      <c r="R14" s="14"/>
+      <c r="S14" s="14"/>
+      <c r="T14" s="14"/>
+      <c r="U14" s="14"/>
+      <c r="V14" s="14"/>
+      <c r="W14" s="14"/>
+      <c r="X14" s="14"/>
+      <c r="Y14" s="14"/>
+      <c r="Z14" s="14"/>
     </row>
     <row r="15" ht="15">
       <c r="B15" s="39"/>
       <c r="C15" s="40"/>
-      <c r="F15" s="40"/>
+      <c r="D15" s="14"/>
+      <c r="E15" s="14"/>
+      <c r="F15" s="41"/>
+      <c r="G15" s="14"/>
+      <c r="H15" s="14"/>
       <c r="I15" s="40"/>
+      <c r="J15" s="14"/>
+      <c r="K15" s="14"/>
       <c r="L15" s="40"/>
+      <c r="M15" s="14"/>
+      <c r="N15" s="14"/>
       <c r="O15" s="40"/>
+      <c r="P15" s="14"/>
+      <c r="Q15" s="14"/>
+      <c r="R15" s="14"/>
+      <c r="S15" s="14"/>
+      <c r="T15" s="14"/>
+      <c r="U15" s="14"/>
+      <c r="V15" s="14"/>
+      <c r="W15" s="14"/>
+      <c r="X15" s="14"/>
+      <c r="Y15" s="14"/>
+      <c r="Z15" s="14"/>
     </row>
     <row r="16" ht="15">
       <c r="B16" s="39"/>
       <c r="C16" s="40"/>
-      <c r="F16" s="40"/>
+      <c r="D16" s="14"/>
+      <c r="E16" s="14"/>
+      <c r="F16" s="41"/>
+      <c r="G16" s="14"/>
+      <c r="H16" s="14"/>
       <c r="I16" s="40"/>
+      <c r="J16" s="14"/>
+      <c r="K16" s="14"/>
       <c r="L16" s="40"/>
+      <c r="M16" s="14"/>
+      <c r="N16" s="14"/>
       <c r="O16" s="40"/>
+      <c r="P16" s="14"/>
+      <c r="Q16" s="14"/>
+      <c r="R16" s="14"/>
+      <c r="S16" s="14"/>
+      <c r="T16" s="14"/>
+      <c r="U16" s="14"/>
+      <c r="V16" s="14"/>
+      <c r="W16" s="14"/>
+      <c r="X16" s="14"/>
+      <c r="Y16" s="14"/>
+      <c r="Z16" s="14"/>
     </row>
     <row r="17" ht="15">
       <c r="B17" s="39"/>
       <c r="C17" s="40"/>
-      <c r="F17" s="40"/>
+      <c r="D17" s="14"/>
+      <c r="E17" s="14"/>
+      <c r="F17" s="41"/>
+      <c r="G17" s="14"/>
+      <c r="H17" s="14"/>
       <c r="I17" s="40"/>
+      <c r="J17" s="14"/>
+      <c r="K17" s="14"/>
       <c r="L17" s="40"/>
+      <c r="M17" s="14"/>
+      <c r="N17" s="14"/>
       <c r="O17" s="40"/>
+      <c r="P17" s="14"/>
+      <c r="Q17" s="14"/>
+      <c r="R17" s="14"/>
+      <c r="S17" s="14"/>
+      <c r="T17" s="14"/>
+      <c r="U17" s="14"/>
+      <c r="V17" s="14"/>
+      <c r="W17" s="14"/>
+      <c r="X17" s="14"/>
+      <c r="Y17" s="14"/>
+      <c r="Z17" s="14"/>
     </row>
     <row r="18" ht="15">
       <c r="B18" s="39"/>
       <c r="C18" s="40"/>
-      <c r="F18" s="40"/>
+      <c r="D18" s="14"/>
+      <c r="E18" s="14"/>
+      <c r="F18" s="41"/>
+      <c r="G18" s="14"/>
+      <c r="H18" s="14"/>
       <c r="I18" s="40"/>
+      <c r="J18" s="14"/>
+      <c r="K18" s="14"/>
       <c r="L18" s="40"/>
+      <c r="M18" s="14"/>
+      <c r="N18" s="14"/>
       <c r="O18" s="40"/>
+      <c r="P18" s="14"/>
+      <c r="Q18" s="14"/>
+      <c r="R18" s="14"/>
+      <c r="S18" s="14"/>
+      <c r="T18" s="14"/>
+      <c r="U18" s="14"/>
+      <c r="V18" s="14"/>
+      <c r="W18" s="14"/>
+      <c r="X18" s="14"/>
+      <c r="Y18" s="14"/>
+      <c r="Z18" s="14"/>
     </row>
     <row r="19" ht="15">
       <c r="B19" s="39"/>
       <c r="C19" s="40"/>
-      <c r="F19" s="40"/>
+      <c r="D19" s="14"/>
+      <c r="E19" s="14"/>
+      <c r="F19" s="41"/>
+      <c r="G19" s="14"/>
+      <c r="H19" s="14"/>
       <c r="I19" s="40"/>
+      <c r="J19" s="14"/>
+      <c r="K19" s="14"/>
       <c r="L19" s="40"/>
+      <c r="M19" s="14"/>
+      <c r="N19" s="14"/>
       <c r="O19" s="40"/>
+      <c r="P19" s="14"/>
+      <c r="Q19" s="14"/>
+      <c r="R19" s="14"/>
+      <c r="S19" s="14"/>
+      <c r="T19" s="14"/>
+      <c r="U19" s="14"/>
+      <c r="V19" s="14"/>
+      <c r="W19" s="14"/>
+      <c r="X19" s="14"/>
+      <c r="Y19" s="14"/>
+      <c r="Z19" s="14"/>
     </row>
     <row r="20" ht="15">
       <c r="B20" s="39"/>
       <c r="C20" s="40"/>
-      <c r="F20" s="40"/>
+      <c r="D20" s="14"/>
+      <c r="E20" s="14"/>
+      <c r="F20" s="41"/>
+      <c r="G20" s="14"/>
+      <c r="H20" s="14"/>
       <c r="I20" s="40"/>
+      <c r="J20" s="14"/>
+      <c r="K20" s="14"/>
       <c r="L20" s="40"/>
+      <c r="M20" s="14"/>
+      <c r="N20" s="14"/>
       <c r="O20" s="40"/>
+      <c r="P20" s="14"/>
+      <c r="Q20" s="14"/>
+      <c r="R20" s="14"/>
+      <c r="S20" s="14"/>
+      <c r="T20" s="14"/>
+      <c r="U20" s="14"/>
+      <c r="V20" s="14"/>
+      <c r="W20" s="14"/>
+      <c r="X20" s="14"/>
+      <c r="Y20" s="14"/>
+      <c r="Z20" s="14"/>
     </row>
     <row r="21" ht="15.75" customHeight="1">
       <c r="B21" s="39"/>
       <c r="C21" s="40"/>
-      <c r="F21" s="40"/>
+      <c r="D21" s="14"/>
+      <c r="E21" s="14"/>
+      <c r="F21" s="41"/>
+      <c r="G21" s="14"/>
+      <c r="H21" s="14"/>
       <c r="I21" s="40"/>
+      <c r="J21" s="14"/>
+      <c r="K21" s="14"/>
       <c r="L21" s="40"/>
+      <c r="M21" s="14"/>
+      <c r="N21" s="14"/>
       <c r="O21" s="40"/>
+      <c r="P21" s="14"/>
+      <c r="Q21" s="14"/>
+      <c r="R21" s="14"/>
+      <c r="S21" s="14"/>
+      <c r="T21" s="14"/>
+      <c r="U21" s="14"/>
+      <c r="V21" s="14"/>
+      <c r="W21" s="14"/>
+      <c r="X21" s="14"/>
+      <c r="Y21" s="14"/>
+      <c r="Z21" s="14"/>
     </row>
     <row r="22" ht="15.75" customHeight="1">
       <c r="B22" s="39"/>
       <c r="C22" s="40"/>
-      <c r="F22" s="40"/>
+      <c r="D22" s="14"/>
+      <c r="E22" s="14"/>
+      <c r="F22" s="41"/>
+      <c r="G22" s="14"/>
+      <c r="H22" s="14"/>
       <c r="I22" s="40"/>
+      <c r="J22" s="14"/>
+      <c r="K22" s="14"/>
       <c r="L22" s="40"/>
+      <c r="M22" s="14"/>
+      <c r="N22" s="14"/>
       <c r="O22" s="40"/>
+      <c r="P22" s="14"/>
+      <c r="Q22" s="14"/>
+      <c r="R22" s="14"/>
+      <c r="S22" s="14"/>
+      <c r="T22" s="14"/>
+      <c r="U22" s="14"/>
+      <c r="V22" s="14"/>
+      <c r="W22" s="14"/>
+      <c r="X22" s="14"/>
+      <c r="Y22" s="14"/>
+      <c r="Z22" s="14"/>
     </row>
     <row r="23" ht="15.75" customHeight="1">
       <c r="B23" s="39"/>
       <c r="C23" s="40"/>
-      <c r="F23" s="40"/>
+      <c r="D23" s="14"/>
+      <c r="E23" s="14"/>
+      <c r="F23" s="41"/>
+      <c r="G23" s="14"/>
+      <c r="H23" s="14"/>
       <c r="I23" s="40"/>
+      <c r="J23" s="14"/>
+      <c r="K23" s="14"/>
       <c r="L23" s="40"/>
+      <c r="M23" s="14"/>
+      <c r="N23" s="14"/>
       <c r="O23" s="40"/>
+      <c r="P23" s="14"/>
+      <c r="Q23" s="14"/>
+      <c r="R23" s="14"/>
+      <c r="S23" s="14"/>
+      <c r="T23" s="14"/>
+      <c r="U23" s="14"/>
+      <c r="V23" s="14"/>
+      <c r="W23" s="14"/>
+      <c r="X23" s="14"/>
+      <c r="Y23" s="14"/>
+      <c r="Z23" s="14"/>
     </row>
     <row r="24" ht="15.75" customHeight="1">
       <c r="B24" s="39"/>
       <c r="C24" s="40"/>
-      <c r="F24" s="40"/>
+      <c r="D24" s="14"/>
+      <c r="E24" s="14"/>
+      <c r="F24" s="41"/>
+      <c r="G24" s="14"/>
+      <c r="H24" s="14"/>
       <c r="I24" s="40"/>
+      <c r="J24" s="14"/>
+      <c r="K24" s="14"/>
       <c r="L24" s="40"/>
+      <c r="M24" s="14"/>
+      <c r="N24" s="14"/>
       <c r="O24" s="40"/>
+      <c r="P24" s="14"/>
+      <c r="Q24" s="14"/>
+      <c r="R24" s="14"/>
+      <c r="S24" s="14"/>
+      <c r="T24" s="14"/>
+      <c r="U24" s="14"/>
+      <c r="V24" s="14"/>
+      <c r="W24" s="14"/>
+      <c r="X24" s="14"/>
+      <c r="Y24" s="14"/>
+      <c r="Z24" s="14"/>
     </row>
     <row r="25" ht="15.75" customHeight="1">
       <c r="B25" s="39"/>
       <c r="C25" s="40"/>
-      <c r="F25" s="40"/>
+      <c r="D25" s="14"/>
+      <c r="E25" s="14"/>
+      <c r="F25" s="41"/>
+      <c r="G25" s="14"/>
+      <c r="H25" s="14"/>
       <c r="I25" s="40"/>
+      <c r="J25" s="14"/>
+      <c r="K25" s="14"/>
       <c r="L25" s="40"/>
+      <c r="M25" s="14"/>
+      <c r="N25" s="14"/>
       <c r="O25" s="40"/>
+      <c r="P25" s="14"/>
+      <c r="Q25" s="14"/>
+      <c r="R25" s="14"/>
+      <c r="S25" s="14"/>
+      <c r="T25" s="14"/>
+      <c r="U25" s="14"/>
+      <c r="V25" s="14"/>
+      <c r="W25" s="14"/>
+      <c r="X25" s="14"/>
+      <c r="Y25" s="14"/>
+      <c r="Z25" s="14"/>
     </row>
     <row r="26" ht="15.75" customHeight="1">
       <c r="B26" s="39"/>
       <c r="C26" s="40"/>
-      <c r="F26" s="40"/>
+      <c r="D26" s="14"/>
+      <c r="E26" s="14"/>
+      <c r="F26" s="41"/>
+      <c r="G26" s="14"/>
+      <c r="H26" s="14"/>
       <c r="I26" s="40"/>
+      <c r="J26" s="14"/>
+      <c r="K26" s="14"/>
       <c r="L26" s="40"/>
+      <c r="M26" s="14"/>
+      <c r="N26" s="14"/>
       <c r="O26" s="40"/>
+      <c r="P26" s="14"/>
+      <c r="Q26" s="14"/>
+      <c r="R26" s="14"/>
+      <c r="S26" s="14"/>
+      <c r="T26" s="14"/>
+      <c r="U26" s="14"/>
+      <c r="V26" s="14"/>
+      <c r="W26" s="14"/>
+      <c r="X26" s="14"/>
+      <c r="Y26" s="14"/>
+      <c r="Z26" s="14"/>
     </row>
     <row r="27" ht="15.75" customHeight="1">
       <c r="B27" s="39"/>
       <c r="C27" s="40"/>
-      <c r="F27" s="40"/>
+      <c r="D27" s="14"/>
+      <c r="E27" s="14"/>
+      <c r="F27" s="41"/>
+      <c r="G27" s="14"/>
+      <c r="H27" s="14"/>
       <c r="I27" s="40"/>
+      <c r="J27" s="14"/>
+      <c r="K27" s="14"/>
       <c r="L27" s="40"/>
+      <c r="M27" s="14"/>
+      <c r="N27" s="14"/>
       <c r="O27" s="40"/>
+      <c r="P27" s="14"/>
+      <c r="Q27" s="14"/>
+      <c r="R27" s="14"/>
+      <c r="S27" s="14"/>
+      <c r="T27" s="14"/>
+      <c r="U27" s="14"/>
+      <c r="V27" s="14"/>
+      <c r="W27" s="14"/>
+      <c r="X27" s="14"/>
+      <c r="Y27" s="14"/>
+      <c r="Z27" s="14"/>
     </row>
     <row r="28" ht="15.75" customHeight="1">
       <c r="B28" s="39"/>
       <c r="C28" s="40"/>
-      <c r="F28" s="40"/>
+      <c r="D28" s="14"/>
+      <c r="E28" s="14"/>
+      <c r="F28" s="41"/>
+      <c r="G28" s="14"/>
+      <c r="H28" s="14"/>
       <c r="I28" s="40"/>
+      <c r="J28" s="14"/>
+      <c r="K28" s="14"/>
       <c r="L28" s="40"/>
+      <c r="M28" s="14"/>
+      <c r="N28" s="14"/>
       <c r="O28" s="40"/>
+      <c r="P28" s="14"/>
+      <c r="Q28" s="14"/>
+      <c r="R28" s="14"/>
+      <c r="S28" s="14"/>
+      <c r="T28" s="14"/>
+      <c r="U28" s="14"/>
+      <c r="V28" s="14"/>
+      <c r="W28" s="14"/>
+      <c r="X28" s="14"/>
+      <c r="Y28" s="14"/>
+      <c r="Z28" s="14"/>
     </row>
     <row r="29" ht="15.75" customHeight="1">
       <c r="B29" s="39"/>
       <c r="C29" s="40"/>
-      <c r="F29" s="40"/>
+      <c r="D29" s="14"/>
+      <c r="E29" s="14"/>
+      <c r="F29" s="41"/>
+      <c r="G29" s="14"/>
+      <c r="H29" s="14"/>
       <c r="I29" s="40"/>
+      <c r="J29" s="14"/>
+      <c r="K29" s="14"/>
       <c r="L29" s="40"/>
+      <c r="M29" s="14"/>
+      <c r="N29" s="14"/>
       <c r="O29" s="40"/>
+      <c r="P29" s="14"/>
+      <c r="Q29" s="14"/>
+      <c r="R29" s="14"/>
+      <c r="S29" s="14"/>
+      <c r="T29" s="14"/>
+      <c r="U29" s="14"/>
+      <c r="V29" s="14"/>
+      <c r="W29" s="14"/>
+      <c r="X29" s="14"/>
+      <c r="Y29" s="14"/>
+      <c r="Z29" s="14"/>
     </row>
     <row r="30" ht="15.75" customHeight="1">
       <c r="B30" s="39"/>
       <c r="C30" s="40"/>
-      <c r="F30" s="40"/>
+      <c r="D30" s="14"/>
+      <c r="E30" s="14"/>
+      <c r="F30" s="41"/>
+      <c r="G30" s="14"/>
+      <c r="H30" s="14"/>
       <c r="I30" s="40"/>
+      <c r="J30" s="14"/>
+      <c r="K30" s="14"/>
       <c r="L30" s="40"/>
+      <c r="M30" s="14"/>
+      <c r="N30" s="14"/>
       <c r="O30" s="40"/>
+      <c r="P30" s="14"/>
+      <c r="Q30" s="14"/>
+      <c r="R30" s="14"/>
+      <c r="S30" s="14"/>
+      <c r="T30" s="14"/>
+      <c r="U30" s="14"/>
+      <c r="V30" s="14"/>
+      <c r="W30" s="14"/>
+      <c r="X30" s="14"/>
+      <c r="Y30" s="14"/>
+      <c r="Z30" s="14"/>
     </row>
     <row r="31" ht="15.75" customHeight="1">
       <c r="B31" s="39"/>
       <c r="C31" s="40"/>
-      <c r="F31" s="40"/>
+      <c r="D31" s="14"/>
+      <c r="E31" s="14"/>
+      <c r="F31" s="41"/>
+      <c r="G31" s="14"/>
+      <c r="H31" s="14"/>
       <c r="I31" s="40"/>
+      <c r="J31" s="14"/>
+      <c r="K31" s="14"/>
       <c r="L31" s="40"/>
+      <c r="M31" s="14"/>
+      <c r="N31" s="14"/>
       <c r="O31" s="40"/>
+      <c r="P31" s="14"/>
+      <c r="Q31" s="14"/>
+      <c r="R31" s="14"/>
+      <c r="S31" s="14"/>
+      <c r="T31" s="14"/>
+      <c r="U31" s="14"/>
+      <c r="V31" s="14"/>
+      <c r="W31" s="14"/>
+      <c r="X31" s="14"/>
+      <c r="Y31" s="14"/>
+      <c r="Z31" s="14"/>
     </row>
     <row r="32" ht="15.75" customHeight="1">
       <c r="B32" s="39"/>
       <c r="C32" s="40"/>
-      <c r="F32" s="40"/>
+      <c r="D32" s="14"/>
+      <c r="E32" s="14"/>
+      <c r="F32" s="41"/>
+      <c r="G32" s="14"/>
+      <c r="H32" s="14"/>
       <c r="I32" s="40"/>
+      <c r="J32" s="14"/>
+      <c r="K32" s="14"/>
       <c r="L32" s="40"/>
+      <c r="M32" s="14"/>
+      <c r="N32" s="14"/>
       <c r="O32" s="40"/>
+      <c r="P32" s="14"/>
+      <c r="Q32" s="14"/>
+      <c r="R32" s="14"/>
+      <c r="S32" s="14"/>
+      <c r="T32" s="14"/>
+      <c r="U32" s="14"/>
+      <c r="V32" s="14"/>
+      <c r="W32" s="14"/>
+      <c r="X32" s="14"/>
+      <c r="Y32" s="14"/>
+      <c r="Z32" s="14"/>
     </row>
     <row r="33" ht="15.75" customHeight="1">
       <c r="B33" s="39"/>
       <c r="C33" s="40"/>
-      <c r="F33" s="40"/>
+      <c r="D33" s="14"/>
+      <c r="E33" s="14"/>
+      <c r="F33" s="41"/>
+      <c r="G33" s="14"/>
+      <c r="H33" s="14"/>
       <c r="I33" s="40"/>
+      <c r="J33" s="14"/>
+      <c r="K33" s="14"/>
       <c r="L33" s="40"/>
+      <c r="M33" s="14"/>
+      <c r="N33" s="14"/>
       <c r="O33" s="40"/>
+      <c r="P33" s="14"/>
+      <c r="Q33" s="14"/>
+      <c r="R33" s="14"/>
+      <c r="S33" s="14"/>
+      <c r="T33" s="14"/>
+      <c r="U33" s="14"/>
+      <c r="V33" s="14"/>
+      <c r="W33" s="14"/>
+      <c r="X33" s="14"/>
+      <c r="Y33" s="14"/>
+      <c r="Z33" s="14"/>
     </row>
     <row r="34" ht="15.75" customHeight="1">
       <c r="B34" s="39"/>
       <c r="C34" s="40"/>
-      <c r="F34" s="40"/>
+      <c r="D34" s="14"/>
+      <c r="E34" s="14"/>
+      <c r="F34" s="41"/>
+      <c r="G34" s="14"/>
+      <c r="H34" s="14"/>
       <c r="I34" s="40"/>
+      <c r="J34" s="14"/>
+      <c r="K34" s="14"/>
       <c r="L34" s="40"/>
+      <c r="M34" s="14"/>
+      <c r="N34" s="14"/>
       <c r="O34" s="40"/>
+      <c r="P34" s="14"/>
+      <c r="Q34" s="14"/>
+      <c r="R34" s="14"/>
+      <c r="S34" s="14"/>
+      <c r="T34" s="14"/>
+      <c r="U34" s="14"/>
+      <c r="V34" s="14"/>
+      <c r="W34" s="14"/>
+      <c r="X34" s="14"/>
+      <c r="Y34" s="14"/>
+      <c r="Z34" s="14"/>
     </row>
     <row r="35" ht="15.75" customHeight="1">
       <c r="B35" s="39"/>
       <c r="C35" s="40"/>
-      <c r="F35" s="40"/>
+      <c r="D35" s="14"/>
+      <c r="E35" s="14"/>
+      <c r="F35" s="41"/>
+      <c r="G35" s="14"/>
+      <c r="H35" s="14"/>
       <c r="I35" s="40"/>
+      <c r="J35" s="14"/>
+      <c r="K35" s="14"/>
       <c r="L35" s="40"/>
+      <c r="M35" s="14"/>
+      <c r="N35" s="14"/>
       <c r="O35" s="40"/>
+      <c r="P35" s="14"/>
+      <c r="Q35" s="14"/>
+      <c r="R35" s="14"/>
+      <c r="S35" s="14"/>
+      <c r="T35" s="14"/>
+      <c r="U35" s="14"/>
+      <c r="V35" s="14"/>
+      <c r="W35" s="14"/>
+      <c r="X35" s="14"/>
+      <c r="Y35" s="14"/>
+      <c r="Z35" s="14"/>
     </row>
     <row r="36" ht="15.75" customHeight="1">
       <c r="B36" s="39"/>
       <c r="C36" s="40"/>
-      <c r="F36" s="40"/>
+      <c r="D36" s="14"/>
+      <c r="E36" s="14"/>
+      <c r="F36" s="41"/>
+      <c r="G36" s="14"/>
+      <c r="H36" s="14"/>
       <c r="I36" s="40"/>
+      <c r="J36" s="14"/>
+      <c r="K36" s="14"/>
       <c r="L36" s="40"/>
+      <c r="M36" s="14"/>
+      <c r="N36" s="14"/>
       <c r="O36" s="40"/>
+      <c r="P36" s="14"/>
+      <c r="Q36" s="14"/>
+      <c r="R36" s="14"/>
+      <c r="S36" s="14"/>
+      <c r="T36" s="14"/>
+      <c r="U36" s="14"/>
+      <c r="V36" s="14"/>
+      <c r="W36" s="14"/>
+      <c r="X36" s="14"/>
+      <c r="Y36" s="14"/>
+      <c r="Z36" s="14"/>
     </row>
     <row r="37" ht="15.75" customHeight="1">
       <c r="B37" s="39"/>
       <c r="C37" s="40"/>
-      <c r="F37" s="40"/>
+      <c r="D37" s="14"/>
+      <c r="E37" s="14"/>
+      <c r="F37" s="41"/>
+      <c r="G37" s="14"/>
+      <c r="H37" s="14"/>
       <c r="I37" s="40"/>
+      <c r="J37" s="14"/>
+      <c r="K37" s="14"/>
       <c r="L37" s="40"/>
+      <c r="M37" s="14"/>
+      <c r="N37" s="14"/>
       <c r="O37" s="40"/>
+      <c r="P37" s="14"/>
+      <c r="Q37" s="14"/>
+      <c r="R37" s="14"/>
+      <c r="S37" s="14"/>
+      <c r="T37" s="14"/>
+      <c r="U37" s="14"/>
+      <c r="V37" s="14"/>
+      <c r="W37" s="14"/>
+      <c r="X37" s="14"/>
+      <c r="Y37" s="14"/>
+      <c r="Z37" s="14"/>
     </row>
     <row r="38" ht="15.75" customHeight="1">
       <c r="B38" s="39"/>
       <c r="C38" s="40"/>
-      <c r="F38" s="40"/>
+      <c r="D38" s="14"/>
+      <c r="E38" s="14"/>
+      <c r="F38" s="41"/>
+      <c r="G38" s="14"/>
+      <c r="H38" s="14"/>
       <c r="I38" s="40"/>
+      <c r="J38" s="14"/>
+      <c r="K38" s="14"/>
       <c r="L38" s="40"/>
+      <c r="M38" s="14"/>
+      <c r="N38" s="14"/>
       <c r="O38" s="40"/>
+      <c r="P38" s="14"/>
+      <c r="Q38" s="14"/>
+      <c r="R38" s="14"/>
+      <c r="S38" s="14"/>
+      <c r="T38" s="14"/>
+      <c r="U38" s="14"/>
+      <c r="V38" s="14"/>
+      <c r="W38" s="14"/>
+      <c r="X38" s="14"/>
+      <c r="Y38" s="14"/>
+      <c r="Z38" s="14"/>
     </row>
     <row r="39" ht="15.75" customHeight="1">
       <c r="B39" s="39"/>
       <c r="C39" s="40"/>
-      <c r="F39" s="40"/>
+      <c r="D39" s="14"/>
+      <c r="E39" s="14"/>
+      <c r="F39" s="41"/>
+      <c r="G39" s="14"/>
+      <c r="H39" s="14"/>
       <c r="I39" s="40"/>
+      <c r="J39" s="14"/>
+      <c r="K39" s="14"/>
       <c r="L39" s="40"/>
+      <c r="M39" s="14"/>
+      <c r="N39" s="14"/>
       <c r="O39" s="40"/>
+      <c r="P39" s="14"/>
+      <c r="Q39" s="14"/>
+      <c r="R39" s="14"/>
+      <c r="S39" s="14"/>
+      <c r="T39" s="14"/>
+      <c r="U39" s="14"/>
+      <c r="V39" s="14"/>
+      <c r="W39" s="14"/>
+      <c r="X39" s="14"/>
+      <c r="Y39" s="14"/>
+      <c r="Z39" s="14"/>
     </row>
     <row r="40" ht="15.75" customHeight="1">
       <c r="B40" s="39"/>
       <c r="C40" s="40"/>
-      <c r="F40" s="40"/>
+      <c r="D40" s="14"/>
+      <c r="E40" s="14"/>
+      <c r="F40" s="41"/>
+      <c r="G40" s="14"/>
+      <c r="H40" s="14"/>
       <c r="I40" s="40"/>
+      <c r="J40" s="14"/>
+      <c r="K40" s="14"/>
       <c r="L40" s="40"/>
+      <c r="M40" s="14"/>
+      <c r="N40" s="14"/>
       <c r="O40" s="40"/>
+      <c r="P40" s="14"/>
+      <c r="Q40" s="14"/>
+      <c r="R40" s="14"/>
+      <c r="S40" s="14"/>
+      <c r="T40" s="14"/>
+      <c r="U40" s="14"/>
+      <c r="V40" s="14"/>
+      <c r="W40" s="14"/>
+      <c r="X40" s="14"/>
+      <c r="Y40" s="14"/>
+      <c r="Z40" s="14"/>
     </row>
     <row r="41" ht="15.75" customHeight="1">
       <c r="B41" s="39"/>
       <c r="C41" s="40"/>
-      <c r="F41" s="40"/>
+      <c r="D41" s="14"/>
+      <c r="E41" s="14"/>
+      <c r="F41" s="41"/>
+      <c r="G41" s="14"/>
+      <c r="H41" s="14"/>
       <c r="I41" s="40"/>
+      <c r="J41" s="14"/>
+      <c r="K41" s="14"/>
       <c r="L41" s="40"/>
+      <c r="M41" s="14"/>
+      <c r="N41" s="14"/>
       <c r="O41" s="40"/>
-    </row>
-    <row r="42" ht="15.75" customHeight="1"/>
-    <row r="43" ht="15.75" customHeight="1"/>
-    <row r="44" ht="15.75" customHeight="1"/>
-    <row r="45" ht="15.75" customHeight="1"/>
-    <row r="46" ht="15.75" customHeight="1"/>
-    <row r="47" ht="15.75" customHeight="1"/>
-    <row r="48" ht="15.75" customHeight="1"/>
-    <row r="49" ht="15.75" customHeight="1"/>
-    <row r="50" ht="15.75" customHeight="1"/>
-    <row r="51" ht="15.75" customHeight="1"/>
-    <row r="52" ht="15.75" customHeight="1"/>
-    <row r="53" ht="15.75" customHeight="1"/>
-    <row r="54" ht="15.75" customHeight="1"/>
+      <c r="P41" s="14"/>
+      <c r="Q41" s="14"/>
+      <c r="R41" s="14"/>
+      <c r="S41" s="14"/>
+      <c r="T41" s="14"/>
+      <c r="U41" s="14"/>
+      <c r="V41" s="14"/>
+      <c r="W41" s="14"/>
+      <c r="X41" s="14"/>
+      <c r="Y41" s="14"/>
+      <c r="Z41" s="14"/>
+    </row>
+    <row r="42" ht="15.75" customHeight="1">
+      <c r="B42" s="14"/>
+      <c r="C42" s="14"/>
+      <c r="D42" s="14"/>
+      <c r="E42" s="14"/>
+      <c r="F42" s="42"/>
+      <c r="G42" s="14"/>
+      <c r="H42" s="14"/>
+      <c r="I42" s="14"/>
+      <c r="J42" s="14"/>
+      <c r="K42" s="14"/>
+      <c r="L42" s="14"/>
+      <c r="M42" s="14"/>
+      <c r="N42" s="14"/>
+      <c r="O42" s="14"/>
+      <c r="P42" s="14"/>
+      <c r="Q42" s="14"/>
+      <c r="R42" s="14"/>
+      <c r="S42" s="14"/>
+      <c r="T42" s="14"/>
+      <c r="U42" s="14"/>
+      <c r="V42" s="14"/>
+      <c r="W42" s="14"/>
+      <c r="X42" s="14"/>
+      <c r="Y42" s="14"/>
+      <c r="Z42" s="14"/>
+    </row>
+    <row r="43" ht="15.75" customHeight="1">
+      <c r="B43" s="14"/>
+      <c r="C43" s="14"/>
+      <c r="D43" s="14"/>
+      <c r="E43" s="14"/>
+      <c r="F43" s="14"/>
+      <c r="G43" s="14"/>
+      <c r="H43" s="14"/>
+      <c r="I43" s="14"/>
+      <c r="J43" s="14"/>
+      <c r="K43" s="14"/>
+      <c r="L43" s="14"/>
+      <c r="M43" s="14"/>
+      <c r="N43" s="14"/>
+      <c r="O43" s="14"/>
+      <c r="P43" s="14"/>
+      <c r="Q43" s="14"/>
+      <c r="R43" s="14"/>
+      <c r="S43" s="14"/>
+      <c r="T43" s="14"/>
+      <c r="U43" s="14"/>
+      <c r="V43" s="14"/>
+      <c r="W43" s="14"/>
+      <c r="X43" s="14"/>
+      <c r="Y43" s="14"/>
+      <c r="Z43" s="14"/>
+    </row>
+    <row r="44" ht="15.75" customHeight="1">
+      <c r="B44" s="14"/>
+      <c r="C44" s="14"/>
+      <c r="D44" s="14"/>
+      <c r="E44" s="14"/>
+      <c r="F44" s="14"/>
+      <c r="G44" s="14"/>
+      <c r="H44" s="14"/>
+      <c r="I44" s="14"/>
+      <c r="J44" s="14"/>
+      <c r="K44" s="14"/>
+      <c r="L44" s="14"/>
+      <c r="M44" s="14"/>
+      <c r="N44" s="14"/>
+      <c r="O44" s="14"/>
+      <c r="P44" s="14"/>
+      <c r="Q44" s="14"/>
+      <c r="R44" s="14"/>
+      <c r="S44" s="14"/>
+      <c r="T44" s="14"/>
+      <c r="U44" s="14"/>
+      <c r="V44" s="14"/>
+      <c r="W44" s="14"/>
+      <c r="X44" s="14"/>
+      <c r="Y44" s="14"/>
+      <c r="Z44" s="14"/>
+    </row>
+    <row r="45" ht="15.75" customHeight="1">
+      <c r="B45" s="14"/>
+      <c r="C45" s="14"/>
+      <c r="D45" s="14"/>
+      <c r="E45" s="14"/>
+      <c r="F45" s="14"/>
+      <c r="G45" s="14"/>
+      <c r="H45" s="14"/>
+      <c r="I45" s="14"/>
+      <c r="J45" s="14"/>
+      <c r="K45" s="14"/>
+      <c r="L45" s="14"/>
+      <c r="M45" s="14"/>
+      <c r="N45" s="14"/>
+      <c r="O45" s="14"/>
+      <c r="P45" s="14"/>
+      <c r="Q45" s="14"/>
+      <c r="R45" s="14"/>
+      <c r="S45" s="14"/>
+      <c r="T45" s="14"/>
+      <c r="U45" s="14"/>
+      <c r="V45" s="14"/>
+      <c r="W45" s="14"/>
+      <c r="X45" s="14"/>
+      <c r="Y45" s="14"/>
+      <c r="Z45" s="14"/>
+    </row>
+    <row r="46" ht="15.75" customHeight="1">
+      <c r="B46" s="14"/>
+      <c r="C46" s="14"/>
+      <c r="D46" s="14"/>
+      <c r="E46" s="14"/>
+      <c r="F46" s="14"/>
+      <c r="G46" s="14"/>
+      <c r="H46" s="14"/>
+      <c r="I46" s="14"/>
+      <c r="J46" s="14"/>
+      <c r="K46" s="14"/>
+      <c r="L46" s="14"/>
+      <c r="M46" s="14"/>
+      <c r="N46" s="14"/>
+      <c r="O46" s="14"/>
+      <c r="P46" s="14"/>
+      <c r="Q46" s="14"/>
+      <c r="R46" s="14"/>
+      <c r="S46" s="14"/>
+      <c r="T46" s="14"/>
+      <c r="U46" s="14"/>
+      <c r="V46" s="14"/>
+      <c r="W46" s="14"/>
+      <c r="X46" s="14"/>
+      <c r="Y46" s="14"/>
+      <c r="Z46" s="14"/>
+    </row>
+    <row r="47" ht="15.75" customHeight="1">
+      <c r="B47" s="14"/>
+      <c r="C47" s="14"/>
+      <c r="D47" s="14"/>
+      <c r="E47" s="14"/>
+      <c r="F47" s="14"/>
+      <c r="G47" s="14"/>
+      <c r="H47" s="14"/>
+      <c r="I47" s="14"/>
+      <c r="J47" s="14"/>
+      <c r="K47" s="14"/>
+      <c r="L47" s="14"/>
+      <c r="M47" s="14"/>
+      <c r="N47" s="14"/>
+      <c r="O47" s="14"/>
+      <c r="P47" s="14"/>
+      <c r="Q47" s="14"/>
+      <c r="R47" s="14"/>
+      <c r="S47" s="14"/>
+      <c r="T47" s="14"/>
+      <c r="U47" s="14"/>
+      <c r="V47" s="14"/>
+      <c r="W47" s="14"/>
+      <c r="X47" s="14"/>
+      <c r="Y47" s="14"/>
+      <c r="Z47" s="14"/>
+    </row>
+    <row r="48" ht="15.75" customHeight="1">
+      <c r="B48" s="14"/>
+      <c r="C48" s="14"/>
+      <c r="D48" s="14"/>
+      <c r="E48" s="14"/>
+      <c r="F48" s="14"/>
+      <c r="G48" s="14"/>
+      <c r="H48" s="14"/>
+      <c r="I48" s="14"/>
+      <c r="J48" s="14"/>
+      <c r="K48" s="14"/>
+      <c r="L48" s="14"/>
+      <c r="M48" s="14"/>
+      <c r="N48" s="14"/>
+      <c r="O48" s="14"/>
+      <c r="P48" s="14"/>
+      <c r="Q48" s="14"/>
+      <c r="R48" s="14"/>
+      <c r="S48" s="14"/>
+      <c r="T48" s="14"/>
+      <c r="U48" s="14"/>
+      <c r="V48" s="14"/>
+      <c r="W48" s="14"/>
+      <c r="X48" s="14"/>
+      <c r="Y48" s="14"/>
+      <c r="Z48" s="14"/>
+    </row>
+    <row r="49" ht="15.75" customHeight="1">
+      <c r="B49" s="14"/>
+      <c r="C49" s="14"/>
+      <c r="D49" s="14"/>
+      <c r="E49" s="14"/>
+      <c r="F49" s="14"/>
+      <c r="G49" s="14"/>
+      <c r="H49" s="14"/>
+      <c r="I49" s="14"/>
+      <c r="J49" s="14"/>
+      <c r="K49" s="14"/>
+      <c r="L49" s="14"/>
+      <c r="M49" s="14"/>
+      <c r="N49" s="14"/>
+      <c r="O49" s="14"/>
+      <c r="P49" s="14"/>
+      <c r="Q49" s="14"/>
+      <c r="R49" s="14"/>
+      <c r="S49" s="14"/>
+      <c r="T49" s="14"/>
+      <c r="U49" s="14"/>
+      <c r="V49" s="14"/>
+      <c r="W49" s="14"/>
+      <c r="X49" s="14"/>
+      <c r="Y49" s="14"/>
+      <c r="Z49" s="14"/>
+    </row>
+    <row r="50" ht="15.75" customHeight="1">
+      <c r="B50" s="14"/>
+      <c r="C50" s="14"/>
+      <c r="D50" s="14"/>
+      <c r="E50" s="14"/>
+      <c r="F50" s="14"/>
+      <c r="G50" s="14"/>
+      <c r="H50" s="14"/>
+      <c r="I50" s="14"/>
+      <c r="J50" s="14"/>
+      <c r="K50" s="14"/>
+      <c r="L50" s="14"/>
+      <c r="M50" s="14"/>
+      <c r="N50" s="14"/>
+      <c r="O50" s="14"/>
+      <c r="P50" s="14"/>
+      <c r="Q50" s="14"/>
+      <c r="R50" s="14"/>
+      <c r="S50" s="14"/>
+      <c r="T50" s="14"/>
+      <c r="U50" s="14"/>
+      <c r="V50" s="14"/>
+      <c r="W50" s="14"/>
+      <c r="X50" s="14"/>
+      <c r="Y50" s="14"/>
+      <c r="Z50" s="14"/>
+    </row>
+    <row r="51" ht="15.75" customHeight="1">
+      <c r="B51" s="14"/>
+      <c r="C51" s="14"/>
+      <c r="D51" s="14"/>
+      <c r="E51" s="14"/>
+      <c r="F51" s="14"/>
+      <c r="G51" s="14"/>
+      <c r="H51" s="14"/>
+      <c r="I51" s="14"/>
+      <c r="J51" s="14"/>
+      <c r="K51" s="14"/>
+      <c r="L51" s="14"/>
+      <c r="M51" s="14"/>
+      <c r="N51" s="14"/>
+      <c r="O51" s="14"/>
+      <c r="P51" s="14"/>
+      <c r="Q51" s="14"/>
+      <c r="R51" s="14"/>
+      <c r="S51" s="14"/>
+      <c r="T51" s="14"/>
+      <c r="U51" s="14"/>
+      <c r="V51" s="14"/>
+      <c r="W51" s="14"/>
+      <c r="X51" s="14"/>
+      <c r="Y51" s="14"/>
+      <c r="Z51" s="14"/>
+    </row>
+    <row r="52" ht="15.75" customHeight="1">
+      <c r="B52" s="14"/>
+      <c r="C52" s="14"/>
+      <c r="D52" s="14"/>
+      <c r="E52" s="14"/>
+      <c r="F52" s="14"/>
+      <c r="G52" s="14"/>
+      <c r="H52" s="14"/>
+      <c r="I52" s="14"/>
+      <c r="J52" s="14"/>
+      <c r="K52" s="14"/>
+      <c r="L52" s="14"/>
+      <c r="M52" s="14"/>
+      <c r="N52" s="14"/>
+      <c r="O52" s="14"/>
+      <c r="P52" s="14"/>
+      <c r="Q52" s="14"/>
+      <c r="R52" s="14"/>
+      <c r="S52" s="14"/>
+      <c r="T52" s="14"/>
+      <c r="U52" s="14"/>
+      <c r="V52" s="14"/>
+      <c r="W52" s="14"/>
+      <c r="X52" s="14"/>
+      <c r="Y52" s="14"/>
+      <c r="Z52" s="14"/>
+    </row>
+    <row r="53" ht="15.75" customHeight="1">
+      <c r="B53" s="14"/>
+      <c r="C53" s="14"/>
+      <c r="D53" s="14"/>
+      <c r="E53" s="14"/>
+      <c r="F53" s="14"/>
+      <c r="G53" s="14"/>
+      <c r="H53" s="14"/>
+      <c r="I53" s="14"/>
+      <c r="J53" s="14"/>
+      <c r="K53" s="14"/>
+      <c r="L53" s="14"/>
+      <c r="M53" s="14"/>
+      <c r="N53" s="14"/>
+      <c r="O53" s="14"/>
+      <c r="P53" s="14"/>
+      <c r="Q53" s="14"/>
+      <c r="R53" s="14"/>
+      <c r="S53" s="14"/>
+      <c r="T53" s="14"/>
+      <c r="U53" s="14"/>
+      <c r="V53" s="14"/>
+      <c r="W53" s="14"/>
+      <c r="X53" s="14"/>
+      <c r="Y53" s="14"/>
+      <c r="Z53" s="14"/>
+    </row>
+    <row r="54" ht="15.75" customHeight="1">
+      <c r="B54" s="14"/>
+      <c r="C54" s="14"/>
+      <c r="D54" s="14"/>
+      <c r="E54" s="14"/>
+      <c r="F54" s="14"/>
+      <c r="G54" s="14"/>
+      <c r="H54" s="14"/>
+      <c r="I54" s="14"/>
+      <c r="J54" s="14"/>
+      <c r="K54" s="14"/>
+      <c r="L54" s="14"/>
+      <c r="M54" s="14"/>
+      <c r="N54" s="14"/>
+      <c r="O54" s="14"/>
+      <c r="P54" s="14"/>
+      <c r="Q54" s="14"/>
+      <c r="R54" s="14"/>
+      <c r="S54" s="14"/>
+      <c r="T54" s="14"/>
+      <c r="U54" s="14"/>
+      <c r="V54" s="14"/>
+      <c r="W54" s="14"/>
+      <c r="X54" s="14"/>
+      <c r="Y54" s="14"/>
+      <c r="Z54" s="14"/>
+    </row>
     <row r="55" ht="15.75" customHeight="1"/>
     <row r="56" ht="15.75" customHeight="1"/>
     <row r="57" ht="15.75" customHeight="1"/>

</xml_diff>